<commit_message>
learn access data change value sort data filter data
</commit_message>
<xml_diff>
--- a/PandaS/Files/phitron_student_marks.xlsx
+++ b/PandaS/Files/phitron_student_marks.xlsx
@@ -478,41 +478,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PH1001</t>
+          <t>94</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alif Rahman</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>85</v>
-      </c>
-      <c r="D2" t="n">
-        <v>85</v>
-      </c>
-      <c r="E2" t="n">
-        <v>88</v>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>94</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mr. Karim</t>
+          <t>94</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>94</t>
         </is>
       </c>
     </row>

</xml_diff>